<commit_message>
fix: improve cleanup transformer and hero parser for cleaner content
Cleanup transformer improvements:
- Remove input elements (search fields become <p> text in scrape)
- Remove a[href="#"] modal trigger links
- Remove leftover modal text by content matching (Search, Return to Site, etc.)
- Remove video player controls, spacers, scroll anchors, tracking pixels
- Remove cart/search/external-site overlay elements

Hero parser fix:
- Skip empty random-background elements that aren't the main hero
- Look for .background img within .slab-content sibling for bg image

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-semaglutide-content-page.report.xlsx
+++ b/tools/importer/reports/import-semaglutide-content-page.report.xlsx
@@ -52,7 +52,7 @@
     <t>semaglutide-content-page</t>
   </si>
   <si>
-    <t>2026-04-16T10:33:44.737Z</t>
+    <t>2026-04-16T16:18:30.858Z</t>
   </si>
   <si>
     <t>Novo Nordisk medicines containing semaglutide | semaglutide.com</t>
@@ -70,7 +70,7 @@
     <t>semaglutide/patient-safety</t>
   </si>
   <si>
-    <t>2026-04-16T10:33:38.078Z</t>
+    <t>2026-04-16T16:18:25.214Z</t>
   </si>
   <si>
     <t>Semaglutide Patient Safety Updates | semaglutide.com</t>

</xml_diff>